<commit_message>
update to ER 09 sample
</commit_message>
<xml_diff>
--- a/data/raw/GLNPO 2024 Spring/GLNPO 2024 Spring/Erie/D20/Rots/ER 09 D20 Spring 2024 24GE00I54 Rot.xlsx
+++ b/data/raw/GLNPO 2024 Spring/GLNPO 2024 Spring/Erie/D20/Rots/ER 09 D20 Spring 2024 24GE00I54 Rot.xlsx
@@ -1,23 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccm243\Desktop\GLNPO Counts\2024\Spring\Erie\d20\Rot\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\GLNPO Zooplankton Database\data\raw\GLNPO 2024 Spring\GLNPO 2024 Spring\Erie\D20\Rots\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E5D030-92D4-4D0D-8FDB-09D036D4B0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{385109E4-8F02-4870-AA41-0D6A66EFB237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{454FAE66-AE17-45BF-A4FD-8663461A8ACC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$V$88</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1150" r:id="rId2"/>
+    <pivotCache cacheId="0" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -332,14 +335,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2555,7 +2557,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4B50A888-7D89-43B0-AA4A-B5DEC15F1E77}" name="PivotTable2" cacheId="1150" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4B50A888-7D89-43B0-AA4A-B5DEC15F1E77}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="X5:AA11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="22">
     <pivotField showAll="0"/>
@@ -2961,6 +2963,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B01B187-420D-430D-A5E4-050BE53ADF1A}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AA88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3042,7 +3045,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -3416,17 +3419,17 @@
       <c r="X7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="Y7" s="4">
+      <c r="Y7">
         <v>166</v>
       </c>
-      <c r="Z7" s="4">
+      <c r="Z7">
         <v>174</v>
       </c>
-      <c r="AA7" s="4">
+      <c r="AA7">
         <v>340</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -3487,13 +3490,13 @@
       <c r="X8" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="Y8" s="4">
+      <c r="Y8">
         <v>158</v>
       </c>
-      <c r="Z8" s="4">
+      <c r="Z8">
         <v>155</v>
       </c>
-      <c r="AA8" s="4">
+      <c r="AA8">
         <v>313</v>
       </c>
     </row>
@@ -3558,13 +3561,13 @@
       <c r="X9" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="Y9" s="4">
+      <c r="Y9">
         <v>15</v>
       </c>
-      <c r="Z9" s="4">
+      <c r="Z9">
         <v>10</v>
       </c>
-      <c r="AA9" s="4">
+      <c r="AA9">
         <v>25</v>
       </c>
     </row>
@@ -3629,13 +3632,13 @@
       <c r="X10" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="Y10" s="4">
-        <v>23</v>
-      </c>
-      <c r="Z10" s="4">
+      <c r="Y10">
+        <v>23</v>
+      </c>
+      <c r="Z10">
         <v>29</v>
       </c>
-      <c r="AA10" s="4">
+      <c r="AA10">
         <v>52</v>
       </c>
     </row>
@@ -3700,13 +3703,13 @@
       <c r="X11" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Y11" s="4">
+      <c r="Y11">
         <v>362</v>
       </c>
-      <c r="Z11" s="4">
+      <c r="Z11">
         <v>368</v>
       </c>
-      <c r="AA11" s="4">
+      <c r="AA11">
         <v>730</v>
       </c>
     </row>
@@ -3769,7 +3772,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -3886,17 +3889,17 @@
       <c r="U14">
         <v>1</v>
       </c>
-      <c r="X14" s="5" t="s">
+      <c r="X14" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="Y14" s="6" t="s">
+      <c r="Y14" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="Z14" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="Z14" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -3954,15 +3957,15 @@
       <c r="U15">
         <v>1</v>
       </c>
-      <c r="X15" s="8"/>
-      <c r="Y15" s="6" t="s">
+      <c r="X15" s="7"/>
+      <c r="Y15" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="Z15" s="7">
+      <c r="Z15" s="6">
         <v>0.999</v>
       </c>
     </row>
-    <row r="16" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -4020,13 +4023,13 @@
       <c r="U16">
         <v>1</v>
       </c>
-      <c r="X16" s="5" t="s">
+      <c r="X16" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="Y16" s="6" t="s">
+      <c r="Y16" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="Z16" s="7">
+      <c r="Z16" s="6">
         <v>1.0029999999999999</v>
       </c>
     </row>
@@ -4088,11 +4091,11 @@
       <c r="U17">
         <v>1</v>
       </c>
-      <c r="X17" s="8"/>
-      <c r="Y17" s="6" t="s">
+      <c r="X17" s="7"/>
+      <c r="Y17" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="Z17" s="7">
+      <c r="Z17" s="6">
         <v>1</v>
       </c>
     </row>
@@ -4154,15 +4157,15 @@
       <c r="U18">
         <v>1</v>
       </c>
-      <c r="X18" s="9" t="s">
+      <c r="X18" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="Y18" s="10" t="s">
+      <c r="Y18" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="Z18" s="11"/>
-    </row>
-    <row r="19" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="Z18" s="10"/>
+    </row>
+    <row r="19" spans="1:26" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -4220,13 +4223,13 @@
       <c r="U19">
         <v>1</v>
       </c>
-      <c r="X19" s="9" t="s">
+      <c r="X19" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="Y19" s="10" t="s">
+      <c r="Y19" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="Z19" s="11"/>
+      <c r="Z19" s="10"/>
     </row>
     <row r="20" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -4286,13 +4289,13 @@
       <c r="U20">
         <v>1</v>
       </c>
-      <c r="X20" s="6" t="s">
+      <c r="X20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="Y20" s="10"/>
-      <c r="Z20" s="11"/>
-    </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y20" s="9"/>
+      <c r="Z20" s="10"/>
+    </row>
+    <row r="21" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -4351,7 +4354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -4410,7 +4413,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -4469,7 +4472,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -4587,7 +4590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>22</v>
       </c>
@@ -4646,7 +4649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>22</v>
       </c>
@@ -4705,7 +4708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -4941,7 +4944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -5000,7 +5003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>22</v>
       </c>
@@ -5118,7 +5121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>22</v>
       </c>
@@ -5413,7 +5416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>22</v>
       </c>
@@ -5531,7 +5534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -5590,7 +5593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>22</v>
       </c>
@@ -5649,7 +5652,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -5708,7 +5711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>22</v>
       </c>
@@ -5767,7 +5770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>22</v>
       </c>
@@ -5885,7 +5888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>22</v>
       </c>
@@ -6239,7 +6242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -6298,7 +6301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>22</v>
       </c>
@@ -6357,7 +6360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>22</v>
       </c>
@@ -6475,7 +6478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>22</v>
       </c>
@@ -6593,7 +6596,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>22</v>
       </c>
@@ -6652,7 +6655,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>22</v>
       </c>
@@ -6770,7 +6773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -7242,7 +7245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>22</v>
       </c>
@@ -7301,7 +7304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>22</v>
       </c>
@@ -7360,7 +7363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -7419,7 +7422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>22</v>
       </c>
@@ -7478,7 +7481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>22</v>
       </c>
@@ -7655,7 +7658,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>22</v>
       </c>
@@ -7752,10 +7755,10 @@
         <v>28</v>
       </c>
       <c r="O79" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="P79" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="Q79" t="s">
         <v>36</v>
@@ -7773,7 +7776,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>22</v>
       </c>
@@ -7832,7 +7835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>22</v>
       </c>
@@ -7891,7 +7894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>22</v>
       </c>
@@ -7950,7 +7953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>22</v>
       </c>
@@ -8009,7 +8012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>22</v>
       </c>
@@ -8127,7 +8130,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="86" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>22</v>
       </c>
@@ -8245,7 +8248,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="88" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>22</v>
       </c>
@@ -8305,6 +8308,14 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:V88" xr:uid="{9B01B187-420D-430D-A5E4-050BE53ADF1A}">
+    <filterColumn colId="17">
+      <filters>
+        <filter val="Copepod nauplii"/>
+        <filter val="Synchaeta spp."/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>